<commit_message>
Improve attribute fill rate: infer specs→options, batch AI, fuzzy match
- Map color_count/品名/规格列 to official options locally (e.g. 12色→colored, HB→hardness)
- Send all unfilled required attrs to AI; relax gate for official attrs (not price/brand)
- Enrich facts_for_ai with text_blob and labeled specs; dedupe red issues
- Regenerate samples/ai_filled_demo.xlsx (colored pencil 0 red issues)

Co-authored-by: nihao555-hub <nihao555-hub@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/icbu-listing/samples/ai_filled_demo.xlsx
+++ b/icbu-listing/samples/ai_filled_demo.xlsx
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -920,27 +920,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>saleProp</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>p-191288435</t>
+          <t>p-191288433</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lead Hardness</t>
+          <t>Lead Color</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>["3460182"]</t>
+          <t>["12970290"]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>colored</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -950,17 +950,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>color_count=12</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>缺依据/待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -977,27 +977,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>saleProp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>p-191288435</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Product name</t>
+          <t>Lead Hardness</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>["3460182"]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>HB</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>HB</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1034,27 +1034,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>saleProp</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>p-200307261</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
+          <t>Number of Colors</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>["44476017"]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>12 Colors</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1067,7 +1067,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>色数 12</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>已填</t>
@@ -1092,22 +1096,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Product name</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Wholesale 12色木杆彩色铅笔</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>Wholesale 12色木杆彩色铅笔</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1117,10 +1121,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Wholesale 12色木杆彩色铅笔</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>已填</t>
@@ -1145,27 +1153,27 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>Minimum order quantity (MOQ)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>500</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>500</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1198,22 +1206,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>阶梯价</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"quantity": "500", "price": "1.80"}</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>500 @ 1.80</t>
+          <t>Piece/Pieces</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1226,11 +1234,7 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>500@1.80</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>已填</t>
@@ -1250,21 +1254,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>p-191288433</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Lead Color</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+          <t>Price setting</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Tiered pricing by quantity</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>是</t>
@@ -1272,17 +1284,13 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -1299,21 +1307,29 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>p-191288433</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Lead Color</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+          <t>阶梯价</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>{"quantity": "500", "price": "1.80"}</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>500 @ 1.80</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>是</t>
@@ -1321,97 +1337,113 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>500@1.80</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PEN-CP-12</t>
+          <t>MKR-WB-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Colored Pencils / 彩色铅笔</t>
+          <t>Art Markers / 美术用马克笔</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>p-191288433</t>
+          <t>p-2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lead Color</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+          <t>Brand Name</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Giorgione</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Giorgione</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>Giorgione</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PEN-CP-12</t>
+          <t>MKR-WB-24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colored Pencils / 彩色铅笔</t>
+          <t>Art Markers / 美术用马克笔</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>p-191288435</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lead Hardness</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+          <t>Place of Origin</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>100000458</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>是</t>
@@ -1419,17 +1451,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>shop</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>China</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -1451,22 +1483,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>p-2</t>
+          <t>p-390873113</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Brand Name</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Giorgione</t>
+          <t>["3542796"]</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Giorgione</t>
+          <t>PLA</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1476,12 +1508,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>vision</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Giorgione</t>
+          <t>Plastic barrel</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1503,42 +1535,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>saleProp</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>p-1</t>
+          <t>p-200307261</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Place of Origin</t>
+          <t>Number of Colors</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>100000458</t>
+          <t>["62999051"]</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>24 Colors</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>色数 24</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1560,42 +1592,42 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>p-390873113</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Material</t>
+          <t>Product name</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>["3542796"]</t>
+          <t>Wholesale 双头美术马克笔24色</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>PLA</t>
+          <t>Wholesale 双头美术马克笔24色</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>vision</t>
+          <t>user</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Plastic barrel</t>
+          <t>Wholesale 双头美术马克笔24色</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1622,39 +1654,35 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Product name</t>
+          <t>Minimum order quantity (MOQ)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>200</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Wholesale 双头美术马克笔24色</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>已填</t>
@@ -1679,27 +1707,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>Piece/Pieces</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1732,22 +1760,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Price setting</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>Tiered pricing by quantity</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1785,22 +1813,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>阶梯价</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>{"quantity": "200", "price": "3.20"}</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>200 @ 3.20</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1813,7 +1841,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>200@3.20</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>已填</t>
@@ -1833,29 +1865,21 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>p-200001254</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>阶梯价</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>{"quantity": "200", "price": "3.20"}</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>200 @ 3.20</t>
-        </is>
-      </c>
+          <t>Dual-side Writing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>是</t>
@@ -1863,17 +1887,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>200@3.20</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -1895,12 +1919,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>p-200001254</t>
+          <t>p-210190015</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Dual-side Writing</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1917,7 +1941,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1929,80 +1953,96 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MKR-WB-24</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Art Markers / 美术用马克笔</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>p-210190015</t>
+          <t>p-2</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+          <t>Brand Name</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Giorgione</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Giorgione</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>Giorgione</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MKR-WB-24</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Art Markers / 美术用马克笔</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>p-200001254</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Dual-side Writing</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>Place of Origin</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>100000458</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>是</t>
@@ -2010,48 +2050,56 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>shop</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>China</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MKR-WB-24</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Art Markers / 美术用马克笔</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>p-210190015</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+          <t>Product name</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Wholesale 18色固体水彩颜料</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Wholesale 18色固体水彩颜料</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>是</t>
@@ -2059,97 +2107,109 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>user</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>Wholesale 18色固体水彩颜料</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MKR-WB-24</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Art Markers / 美术用马克笔</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>p-200001254</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Dual-side Writing</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+          <t>Minimum order quantity (MOQ)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MKR-WB-24</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Art Markers / 美术用马克笔</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>p-210190015</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Piece/Pieces</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>是</t>
@@ -2157,17 +2217,13 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -2184,32 +2240,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>p-2</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Brand Name</t>
+          <t>Price setting</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Giorgione</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Giorgione</t>
+          <t>Tiered pricing by quantity</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2217,11 +2273,7 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Giorgione</t>
-        </is>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2241,27 +2293,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>p-1</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Place of Origin</t>
+          <t>阶梯价</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>100000458</t>
+          <t>{"quantity": "300", "price": "4.50"}</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>300 @ 4.50</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2271,12 +2323,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>300@4.50</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2298,29 +2350,21 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>p-210190051</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Product name</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Wholesale 18色固体水彩颜料</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Wholesale 18色固体水彩颜料</t>
-        </is>
-      </c>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>是</t>
@@ -2328,17 +2372,17 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Wholesale 18色固体水彩颜料</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -2355,80 +2399,76 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>p-191288010</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+        </is>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>p-191284014</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>material</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>34313717</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>Rattan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2438,10 +2478,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
+          <t>vision</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>PE rattan</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2451,37 +2495,37 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>p-231671682</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>mail packing</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>111689382</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2491,10 +2535,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
+          <t>fact</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2504,52 +2552,52 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>p-100001004</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>阶梯价</t>
+          <t>sofa type</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>{"quantity": "300", "price": "4.50"}</t>
+          <t>3339564</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>300 @ 4.50</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>fact</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>300@4.50</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2561,31 +2609,39 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>p-210190051</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+          <t>place of origin</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>100000458</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>是</t>
@@ -2593,97 +2649,113 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>shop</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>China</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>p-191288010</t>
+          <t>p-400004414</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+          <t>Rattan</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>1982267690</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>UV-Resistant PE Rattan</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>fact</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>UV-Resistant PE Rattan</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>saleProp</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>p-210190051</t>
+          <t>p-210190015</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>["3399503"]</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>是</t>
@@ -2691,48 +2763,56 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>vision</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>Brown</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>p-191288010</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+          <t>Product name</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>是</t>
@@ -2740,97 +2820,109 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>user</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>Wholesale 户外花园PE藤编沙发三件套</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>p-210190051</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
+          <t>Minimum order quantity (MOQ)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>p-191288010</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Piece/Pieces</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>是</t>
@@ -2838,17 +2930,13 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -2865,27 +2953,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>p-191284014</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>material</t>
+          <t>Price setting</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>34313717</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Rattan</t>
+          <t>Tiered pricing by quantity</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2895,14 +2983,10 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>vision</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>PE rattan</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2922,27 +3006,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>p-1</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>place of origin</t>
+          <t>阶梯价</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>100000458</t>
+          <t>{"quantity": "20", "price": "89.00"}</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>20 @ 89.00</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2952,12 +3036,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>20@89.00</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -2979,29 +3063,21 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>saleProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>p-210190015</t>
+          <t>p-234916993</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>color</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>["3399503"]</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Brown</t>
-        </is>
-      </c>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>是</t>
@@ -3009,17 +3085,17 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>vision</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -3036,29 +3112,21 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>p-235983983</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Product name</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
-        </is>
-      </c>
+          <t>design style</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>是</t>
@@ -3066,17 +3134,17 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -3093,80 +3161,76 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>p-191284006</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr"/>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>p-390873113</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>190092752</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>Hepa</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3176,10 +3240,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr"/>
+          <t>vision</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HEPA paper</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr">
         <is>
           <t>已填</t>
@@ -3189,37 +3257,37 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>place of origin</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>100000458</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>China</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3229,10 +3297,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr"/>
+          <t>shop</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="K47" t="inlineStr">
         <is>
           <t>已填</t>
@@ -3242,42 +3314,42 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>p-360946261</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>阶梯价</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>{"quantity": "20", "price": "89.00"}</t>
+          <t>352×478×30mm</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>20 @ 89.00</t>
+          <t>352×478×30mm</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3287,7 +3359,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>20@89.00</t>
+          <t>352×478×30mm</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3299,31 +3371,39 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>p-231671682</t>
+          <t>p-191284008</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>mail packing</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1982271415</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>High-Efficiency HEPA Filter</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>是</t>
@@ -3331,48 +3411,56 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>fact</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>High-Efficiency HEPA Filter</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>p-234916993</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+          <t>Product name</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Wholesale 空气净化器HEPA滤芯</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Wholesale 空气净化器HEPA滤芯</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>是</t>
@@ -3380,97 +3468,109 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>user</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>Wholesale 空气净化器HEPA滤芯</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>p-235983983</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>design style</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+          <t>Minimum order quantity (MOQ)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>p-191284006</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Piece/Pieces</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
           <t>是</t>
@@ -3478,48 +3578,52 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>p-231671682</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>mail packing</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+          <t>Price setting</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Tiered pricing by quantity</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>是</t>
@@ -3527,48 +3631,52 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>p-234916993</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+          <t>阶梯价</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>{"quantity": "100", "price": "6.50"}</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>100 @ 6.50</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>是</t>
@@ -3576,29 +3684,29 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>100@6.50</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3608,12 +3716,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>p-235983983</t>
+          <t>p-210194274</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>design style</t>
+          <t>application</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -3630,7 +3738,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3642,12 +3750,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3657,12 +3765,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>p-191284006</t>
+          <t>p-210196802</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>size</t>
+          <t>power source</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3679,7 +3787,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3691,12 +3799,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>FILTER-HEPA-01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3706,12 +3814,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>p-231671682</t>
+          <t>p-373265001</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>mail packing</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -3728,1099 +3836,10 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
+          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>SOFA-GD-01</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Garden Sofas / 花园沙发</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>p-234916993</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>SOFA-GD-01</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Garden Sofas / 花园沙发</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>p-235983983</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>design style</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>SOFA-GD-01</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Garden Sofas / 花园沙发</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>p-191284006</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>icbuCatProp</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>p-390873113</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>190092752</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Hepa</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>vision</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>HEPA paper</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>icbuCatProp</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>p-1</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>place of origin</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>100000458</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>shop</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>icbuCatProp</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>p-360946261</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>352×478×30mm</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>352×478×30mm</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>352×478×30mm</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>icbuCatProp</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>p-191284008</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>1982271415</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>High-Efficiency HEPA Filter</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>ai</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>High-Efficiency HEPA Filter</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>trade</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>productTitle</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Product name</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>trade</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>minOrderQuantity</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Minimum order quantity (MOQ)</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>trade</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>priceUnit</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Piece/Pieces</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>trade</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>scPrice</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Price setting</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>Tiered pricing by quantity</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>trade</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>ladderPrice_0</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>阶梯价</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>{"quantity": "100", "price": "6.50"}</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>100 @ 6.50</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>100@6.50</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>已填</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>p-210196802</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>power source</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>p-210194274</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>p-373265001</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>p-210196802</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>power source</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>p-210194274</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>p-373265001</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>p-210196802</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>power source</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>p-210194274</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>未填-待人工</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>FILTER-HEPA-01</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>issue</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>p-373265001</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>平台必填属性缺少依据，AI 未填。请补事实或手动选择</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
         <is>
           <t>未填-待人工</t>
         </is>
@@ -4837,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4847,17 +3866,22 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
-    <col width="29" customWidth="1" min="18" max="18"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="25" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="22" max="22"/>
+    <col width="29" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4898,55 +3922,80 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>icbuCatProp.p-191288433</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>saleProp.p-191288435</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>saleProp.p-200307261</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>trade.productTitle</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>trade.minOrderQuantity</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>trade.priceUnit</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>trade.scPrice</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>trade.ladderPrice_0</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-390873113</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-191284014</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>icbuCatProp.p-231671682</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>icbuCatProp.p-100001004</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>icbuCatProp.p-400004414</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>saleProp.p-210190015</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-360946261</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-191284008</t>
         </is>
@@ -4990,39 +4039,52 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>colored</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>HB</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>12 Colors</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>Wholesale 12色木杆彩色铅笔</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Piece/Pieces</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Tiered pricing by quantity</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>500 @ 1.80</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5061,40 +4123,49 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>24 Colors</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Wholesale 双头美术马克笔24色</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Piece/Pieces</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Tiered pricing by quantity</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>200 @ 3.20</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>PLA</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5133,36 +4204,41 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Wholesale 18色固体水彩颜料</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Piece/Pieces</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Tiered pricing by quantity</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>300 @ 4.50</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5197,44 +4273,61 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Wholesale 户外花园PE藤编沙发三件套</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Piece/Pieces</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Tiered pricing by quantity</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>20 @ 89.00</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Rattan</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>UV-Resistant PE Rattan</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5269,44 +4362,49 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
         <is>
           <t>Wholesale 空气净化器HEPA滤芯</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Piece/Pieces</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Tiered pricing by quantity</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>100 @ 6.50</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Hepa</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
         <is>
           <t>352×478×30mm</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>High-Efficiency HEPA Filter</t>
         </is>
@@ -5419,28 +4517,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -5465,10 +4563,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -5477,7 +4575,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
         <v>3</v>
@@ -5511,7 +4609,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>7</v>
@@ -5523,7 +4621,7 @@
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
         <v>3</v>
@@ -5557,28 +4655,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
         <v>3</v>
-      </c>
-      <c r="H5" t="n">
-        <v>12</v>
       </c>
       <c r="I5" t="n">
         <v>7</v>
       </c>
       <c r="J5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" t="n">
         <v>3</v>
-      </c>
-      <c r="K5" t="n">
-        <v>4</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -5603,19 +4701,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>9</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I6" t="n">
         <v>6</v>
@@ -5641,7 +4739,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-18T18:43:09+00:00</t>
+          <t>2026-08-18T18:51:47+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh ai_filled_demo samples after latest certainty-gate test run
Co-authored-by: nihao555-hub <nihao555-hub@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/icbu-listing/samples/ai_filled_demo.xlsx
+++ b/icbu-listing/samples/ai_filled_demo.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{"color_count": "12", "material": "Wood", "hardness": "HB", "size": "17.5cm"}</t>
+          <t>{"color_count": "12", "material": "Wood", "hardness": "HB", "size": "17.5cm", "color": "colored"}</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -729,10 +729,10 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="29" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -893,7 +893,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>color_count=12</t>
+          <t>multicolored</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1049,12 +1049,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>["44476017"]</t>
+          <t>["68739970"]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12 Colors</t>
+          <t>8 Colors</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>色数 12</t>
+          <t>8 Colors</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>vision</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>色数 24</t>
+          <t>24</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1953,39 +1953,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>WC-PAN-18</t>
+          <t>MKR-WB-24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Water Color / 水合颜料</t>
+          <t>Art Markers / 美术用马克笔</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>p-2</t>
+          <t>scImages</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Brand Name</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Giorgione</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Giorgione</t>
-        </is>
-      </c>
+          <t>产品图片</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>否</t>
@@ -1993,17 +1985,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Giorgione</t>
+          <t>至少要一张图片</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -2025,37 +2017,37 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>p-1</t>
+          <t>p-2</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Place of Origin</t>
+          <t>Brand Name</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>100000458</t>
+          <t>Giorgione</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Giorgione</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Giorgione</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2077,27 +2069,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Product name</t>
+          <t>Place of Origin</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Wholesale 18色固体水彩颜料</t>
+          <t>100000458</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Wholesale 18色固体水彩颜料</t>
+          <t>China</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2107,12 +2099,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Wholesale 18色固体水彩颜料</t>
+          <t>China</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2139,35 +2131,39 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
+          <t>Product name</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Wholesale colored pencil set</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2192,27 +2188,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Minimum order quantity (MOQ)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>300</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2245,22 +2241,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>Piece/Pieces</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2298,22 +2294,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>阶梯价</t>
+          <t>Price setting</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>{"quantity": "300", "price": "4.50"}</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>300 @ 4.50</t>
+          <t>Tiered pricing by quantity</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2326,11 +2322,7 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>300@4.50</t>
-        </is>
-      </c>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2350,21 +2342,29 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>p-210190051</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+          <t>阶梯价</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>{"quantity": "300", "price": "4.50"}</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>300 @ 4.50</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>是</t>
@@ -2372,17 +2372,17 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+          <t>300@4.50</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -2404,12 +2404,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>p-191288010</t>
+          <t>p-210190051</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Color</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2438,39 +2438,31 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>p-191284014</t>
+          <t>p-191288010</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>material</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>34313717</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Rattan</t>
-        </is>
-      </c>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>是</t>
@@ -2478,74 +2470,66 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>vision</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>PE rattan</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SOFA-GD-01</t>
+          <t>WC-PAN-18</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Garden Sofas / 花园沙发</t>
+          <t>Water Color / 水合颜料</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>p-231671682</t>
+          <t>scImages</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mail packing</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>111689382</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>产品图片</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>fact</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>至少要一张图片</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -2567,22 +2551,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>p-100001004</t>
+          <t>p-100000801</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>sofa type</t>
+          <t>specific use</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3339564</t>
+          <t>1875814357</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>Garden Sofa</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2592,12 +2576,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>fact</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>Garden Sofa</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2624,37 +2608,37 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>p-1</t>
+          <t>p-100001000</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>place of origin</t>
+          <t>general use</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>100000458</t>
+          <t>428124982</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Outdoor Furniture</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>pieces 3</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2681,37 +2665,37 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>p-400004414</t>
+          <t>p-191284014</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>34313717</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
           <t>Rattan</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>1982267690</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>UV-Resistant PE Rattan</t>
-        </is>
-      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>fact</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>UV-Resistant PE Rattan</t>
+          <t>PE rattan</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2733,27 +2717,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>saleProp</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>p-210190015</t>
+          <t>p-231671682</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>color</t>
+          <t>mail packing</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>["3399503"]</t>
+          <t>111689382</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2763,12 +2747,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>vision</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2790,42 +2774,42 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>p-100001004</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Product name</t>
+          <t>sofa type</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+          <t>3339564</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,32 +2831,32 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
+          <t>place of origin</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>100000458</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>China</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2880,7 +2864,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2900,32 +2888,32 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>p-400004414</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Rattan</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1982267690</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>UV-Resistant PE Rattan</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2933,7 +2921,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>UV-Resistant PE Rattan</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>已填</t>
@@ -2953,27 +2945,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>saleProp</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>p-210190015</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>color</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>["3399503"]</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>Brown</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2986,7 +2978,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr">
         <is>
           <t>已填</t>
@@ -3011,22 +3007,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>阶梯价</t>
+          <t>Product name</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>{"quantity": "20", "price": "89.00"}</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>20 @ 89.00</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3036,12 +3032,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>user</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>20@89.00</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3063,39 +3059,43 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>p-234916993</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+          <t>Minimum order quantity (MOQ)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -3112,21 +3112,29 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>p-235983983</t>
+          <t>priceUnit</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>design style</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Piece/Pieces</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>是</t>
@@ -3134,17 +3142,13 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -3161,21 +3165,29 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>p-191284006</t>
+          <t>scPrice</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+          <t>Price setting</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Tiered pricing by quantity</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>是</t>
@@ -3183,54 +3195,50 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FILTER-HEPA-01</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>p-390873113</t>
+          <t>ladderPrice_0</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Material</t>
+          <t>阶梯价</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>190092752</t>
+          <t>{"quantity": "20", "price": "89.00"}</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Hepa</t>
+          <t>20 @ 89.00</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3240,12 +3248,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>vision</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>HEPA paper</t>
+          <t>20@89.00</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3257,39 +3265,31 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>FILTER-HEPA-01</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>p-1</t>
+          <t>p-234916993</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>place of origin</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>100000458</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>是</t>
@@ -3297,113 +3297,97 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>FILTER-HEPA-01</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>p-360946261</t>
+          <t>p-235983983</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>352×478×30mm</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>352×478×30mm</t>
-        </is>
-      </c>
+          <t>design style</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>352×478×30mm</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>FILTER-HEPA-01</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>icbuCatProp</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>p-191284008</t>
+          <t>p-191284006</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>1982271415</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>High-Efficiency HEPA Filter</t>
-        </is>
-      </c>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>是</t>
@@ -3411,74 +3395,66 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>fact</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>High-Efficiency HEPA Filter</t>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>FILTER-HEPA-01</t>
+          <t>SOFA-GD-01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Air Purifier Parts / 空气净化器零部件</t>
+          <t>Garden Sofas / 花园沙发</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>issue</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>productTitle</t>
+          <t>scImages</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Product name</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
-        </is>
-      </c>
+          <t>产品图片</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
+          <t>至少要一张图片</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>已填</t>
+          <t>未填-待人工</t>
         </is>
       </c>
     </row>
@@ -3495,32 +3471,32 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>minOrderQuantity</t>
+          <t>p-390873113</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Minimum order quantity (MOQ)</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>190092752</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>Hepa</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3528,7 +3504,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>HEPA paper</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>已填</t>
@@ -3548,27 +3528,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>priceUnit</t>
+          <t>p-1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>place of origin</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>100000458</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Piece/Pieces</t>
+          <t>China</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3581,7 +3561,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="K52" t="inlineStr">
         <is>
           <t>已填</t>
@@ -3601,32 +3585,32 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>scPrice</t>
+          <t>p-360946261</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Price setting</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>352×478×30mm</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Tiered pricing by quantity</t>
+          <t>352×478×30mm</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3634,7 +3618,11 @@
           <t>excel</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>352×478×30mm</t>
+        </is>
+      </c>
       <c r="K53" t="inlineStr">
         <is>
           <t>已填</t>
@@ -3654,27 +3642,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>icbuCatProp</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ladderPrice_0</t>
+          <t>p-191284008</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>阶梯价</t>
+          <t>type</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>{"quantity": "100", "price": "6.50"}</t>
+          <t>190092098</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>100 @ 6.50</t>
+          <t>Filter</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3689,7 +3677,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>100@6.50</t>
+          <t>Filter</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3711,21 +3699,29 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>p-210194274</t>
+          <t>productTitle</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>application</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+          <t>Product name</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Wholesale colored pencil set</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Wholesale colored pencil set</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>是</t>
@@ -3733,17 +3729,17 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>user</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -3760,39 +3756,43 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>issue</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>p-210196802</t>
+          <t>minOrderQuantity</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>power source</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
+          <t>Minimum order quantity (MOQ)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
-        </is>
-      </c>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>未填-待人工</t>
+          <t>已填</t>
         </is>
       </c>
     </row>
@@ -3809,37 +3809,347 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
+          <t>trade</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>priceUnit</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Piece/Pieces</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>已填</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>FILTER-HEPA-01</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>trade</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>scPrice</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Price setting</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Tiered pricing by quantity</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>已填</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>FILTER-HEPA-01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>trade</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ladderPrice_0</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>阶梯价</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>{"quantity": "100", "price": "6.50"}</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>100 @ 6.50</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>100@6.50</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>已填</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>FILTER-HEPA-01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
           <t>issue</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>p-210194274</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>application</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>未填-待人工</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>FILTER-HEPA-01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>issue</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>p-210196802</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>power source</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>未填-待人工</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>FILTER-HEPA-01</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>issue</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
         <is>
           <t>p-373265001</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr">
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>平台必填属性仍缺事实依据，请补规格或人工选择</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>平台必填字段无法百分百确定，请补事实或人工填写</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>未填-待人工</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>FILTER-HEPA-01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Air Purifier Parts / 空气净化器零部件</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>issue</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>scImages</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>产品图片</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>至少要一张图片</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t>未填-待人工</t>
         </is>
@@ -3856,12 +4166,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
@@ -3869,7 +4179,7 @@
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="28" customWidth="1" min="14" max="14"/>
@@ -3879,9 +4189,11 @@
     <col width="25" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
     <col width="25" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="25" customWidth="1" min="22" max="22"/>
-    <col width="29" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="25" customWidth="1" min="24" max="24"/>
+    <col width="25" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3967,35 +4279,45 @@
       </c>
       <c r="Q1" s="3" t="inlineStr">
         <is>
+          <t>icbuCatProp.p-100000801</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>icbuCatProp.p-100001000</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
           <t>icbuCatProp.p-191284014</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-231671682</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-100001004</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-400004414</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>saleProp.p-210190015</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-360946261</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>icbuCatProp.p-191284008</t>
         </is>
@@ -4014,7 +4336,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4049,12 +4371,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12 Colors</t>
+          <t>8 Colors</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Wholesale 12色木杆彩色铅笔</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -4085,6 +4407,8 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4099,7 +4423,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4131,7 +4455,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Wholesale 双头美术马克笔24色</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -4166,6 +4490,8 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4180,7 +4506,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wholesale 18色固体水彩颜料</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -4208,7 +4534,7 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Wholesale 18色固体水彩颜料</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -4239,6 +4565,8 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4253,7 +4581,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4277,7 +4605,7 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Wholesale 户外花园PE藤编沙发三件套</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -4303,31 +4631,41 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
+          <t>Garden Sofa</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Outdoor Furniture</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>Rattan</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Set</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>UV-Resistant PE Rattan</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4342,7 +4680,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4366,7 +4704,7 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Wholesale 空气净化器HEPA滤芯</t>
+          <t>Wholesale colored pencil set</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -4399,14 +4737,16 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr">
         <is>
           <t>352×478×30mm</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>High-Efficiency HEPA Filter</t>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Filter</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4765,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -4435,7 +4775,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4542,7 +4882,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>无依据的必填项留空标红，需人工补或补事实后再生成</t>
+          <t>无依据的必填项留空标红；有图时会先 vision 识图再 multimodal 填属性</t>
         </is>
       </c>
     </row>
@@ -4575,7 +4915,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>3</v>
@@ -4588,7 +4928,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>无依据的必填项留空标红，需人工补或补事实后再生成</t>
+          <t>无依据的必填项留空标红；有图时会先 vision 识图再 multimodal 填属性</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4961,7 @@
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>3</v>
@@ -4634,7 +4974,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>无依据的必填项留空标红，需人工补或补事实后再生成</t>
+          <t>无依据的必填项留空标红；有图时会先 vision 识图再 multimodal 填属性</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4998,7 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -4667,7 +5007,7 @@
         <v>4</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I5" t="n">
         <v>7</v>
@@ -4680,7 +5020,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>无依据的必填项留空标红，需人工补或补事实后再生成</t>
+          <t>无依据的必填项留空标红；有图时会先 vision 识图再 multimodal 填属性</t>
         </is>
       </c>
     </row>
@@ -4713,7 +5053,7 @@
         <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
         <v>6</v>
@@ -4726,7 +5066,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>无依据的必填项留空标红，需人工补或补事实后再生成</t>
+          <t>无依据的必填项留空标红；有图时会先 vision 识图再 multimodal 填属性</t>
         </is>
       </c>
     </row>
@@ -4739,7 +5079,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-18T18:51:47+00:00</t>
+          <t>2026-08-18T19:04:08+00:00</t>
         </is>
       </c>
     </row>
@@ -4751,7 +5091,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Excel事实 → AI填官方属性 → 导出（未发布）</t>
+          <t>Excel事实+商品图 → vision识图 → AI填官方属性 → 导出（未发布）</t>
         </is>
       </c>
     </row>

</xml_diff>